<commit_message>
Added data from Weber et al. (2026, ACP)
Mineralogical and morphological data from: Weber, A. M., Kutuzov, S., Beaudon, E., Sierra-Hernández, M. R., Davis, M., Bayless, L. H., Kenny, D., & Thompson, L. G. (2026). Ice core insights into the morphology and composition of mineral dust deposited in the tropical Peruvian Andes. Atmospheric Chemistry and Physics, 26(17), 12887–12909. https://doi.org/10.5194/acp-26-12887-2026
</commit_message>
<xml_diff>
--- a/data/byrd-data-info.xlsx
+++ b/data/byrd-data-info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin Weber\AppData\Roaming\MathWorks\MATLAB Add-Ons\Collections\ByrdDIT - The Byrd Data Import Tool\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin Weber\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D868AA4-F77E-44A9-A223-BB6A307F5D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6A625C0-F154-4330-A508-3D3A4D8C40D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="368" windowWidth="21600" windowHeight="11054" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="publication" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="133">
   <si>
     <t>bona-churchill</t>
   </si>
@@ -394,9 +394,6 @@
     <t>Kinnard et al. (2011b)</t>
   </si>
   <si>
-    <t>Weber et al. (2026)</t>
-  </si>
-  <si>
     <t>2019-dust</t>
   </si>
   <si>
@@ -431,6 +428,15 @@
   </si>
   <si>
     <t>summit-CH4</t>
+  </si>
+  <si>
+    <t>Weber et al. (2026a)</t>
+  </si>
+  <si>
+    <t>Weber et al. (2026b)</t>
+  </si>
+  <si>
+    <t>col-mineralogy</t>
   </si>
 </sst>
 </file>
@@ -823,7 +829,7 @@
         <v>79</v>
       </c>
       <c r="R1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="S1" t="s">
         <v>72</v>
@@ -837,7 +843,7 @@
         <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D2" t="s">
         <v>111</v>
@@ -855,7 +861,7 @@
         <v>97</v>
       </c>
       <c r="I2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J2" t="s">
         <v>100</v>
@@ -867,7 +873,7 @@
         <v>102</v>
       </c>
       <c r="M2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="N2" t="s">
         <v>105</v>
@@ -882,7 +888,7 @@
         <v>109</v>
       </c>
       <c r="R2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="S2" t="s">
         <v>117</v>
@@ -899,7 +905,7 @@
         <v>93</v>
       </c>
       <c r="I3" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="J3" t="s">
         <v>101</v>
@@ -919,7 +925,7 @@
         <v>113</v>
       </c>
       <c r="I4" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="M4" t="s">
         <v>112</v>
@@ -933,7 +939,7 @@
         <v>114</v>
       </c>
       <c r="I5" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.45">
@@ -941,12 +947,15 @@
         <v>92</v>
       </c>
       <c r="I6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.45">
       <c r="F7" t="s">
         <v>94</v>
+      </c>
+      <c r="I7" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.45">
@@ -961,7 +970,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BF50EB8-00C0-4B81-9C39-E2A1C82D00CC}">
-  <dimension ref="A1:AK11"/>
+  <dimension ref="A1:AL11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="25.53125" bestFit="1" customWidth="1"/>
@@ -979,26 +988,26 @@
     <col min="14" max="15" width="19.86328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="31.6640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="20" width="19.86328125" customWidth="1"/>
-    <col min="21" max="21" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.86328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="22" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.46484375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="18.53125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.53125" customWidth="1"/>
-    <col min="28" max="28" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="20.86328125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="30.1328125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="21.796875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="26.6640625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="25.1328125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="25.1328125" customWidth="1"/>
-    <col min="37" max="37" width="18.46484375" bestFit="1" customWidth="1"/>
+    <col min="18" max="21" width="19.86328125" customWidth="1"/>
+    <col min="22" max="22" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="22" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="18.46484375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.53125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="18.53125" customWidth="1"/>
+    <col min="29" max="29" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="20.86328125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="30.1328125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="21.796875" bestFit="1" customWidth="1"/>
+    <col min="33" max="34" width="19.86328125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="25.1328125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="25.1328125" customWidth="1"/>
+    <col min="38" max="38" width="18.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:38" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1066,19 +1075,19 @@
         <v>25</v>
       </c>
       <c r="W1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="X1" t="s">
         <v>36</v>
       </c>
       <c r="Y1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z1" t="s">
         <v>39</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>40</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>48</v>
       </c>
       <c r="AB1" t="s">
         <v>48</v>
@@ -1087,7 +1096,7 @@
         <v>48</v>
       </c>
       <c r="AD1" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="AE1" t="s">
         <v>56</v>
@@ -1096,22 +1105,25 @@
         <v>56</v>
       </c>
       <c r="AG1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AH1" t="s">
         <v>67</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>71</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>79</v>
       </c>
-      <c r="AJ1" t="s">
-        <v>125</v>
-      </c>
       <c r="AK1" t="s">
+        <v>124</v>
+      </c>
+      <c r="AL1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:38" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>110</v>
       </c>
@@ -1122,7 +1134,7 @@
         <v>88</v>
       </c>
       <c r="D2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E2" t="s">
         <v>89</v>
@@ -1164,67 +1176,70 @@
         <v>97</v>
       </c>
       <c r="R2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="S2" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="T2" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="U2" t="s">
+        <v>122</v>
+      </c>
+      <c r="V2" t="s">
         <v>98</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>99</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
         <v>101</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>100</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>116</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" t="s">
         <v>102</v>
       </c>
-      <c r="AA2" t="s">
-        <v>121</v>
-      </c>
       <c r="AB2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AC2" t="s">
         <v>103</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>112</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
         <v>105</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AF2" t="s">
         <v>106</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AG2" t="s">
         <v>104</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AH2" t="s">
         <v>107</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AI2" t="s">
         <v>108</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AJ2" t="s">
         <v>109</v>
       </c>
-      <c r="AJ2" t="s">
-        <v>126</v>
-      </c>
       <c r="AK2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AL2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:38" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1235,7 +1250,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E3" t="s">
         <v>8</v>
@@ -1277,67 +1292,70 @@
         <v>77</v>
       </c>
       <c r="R3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="S3" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="T3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="U3" t="s">
+        <v>123</v>
+      </c>
+      <c r="V3" t="s">
         <v>35</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" t="s">
         <v>26</v>
       </c>
-      <c r="W3" t="s">
+      <c r="X3" t="s">
         <v>38</v>
       </c>
-      <c r="X3" t="s">
+      <c r="Y3" t="s">
         <v>37</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Z3" t="s">
         <v>1</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" t="s">
         <v>41</v>
       </c>
-      <c r="AA3" t="s">
-        <v>122</v>
-      </c>
       <c r="AB3" t="s">
+        <v>121</v>
+      </c>
+      <c r="AC3" t="s">
         <v>8</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AD3" t="s">
         <v>49</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AE3" t="s">
         <v>60</v>
       </c>
-      <c r="AE3" t="s">
+      <c r="AF3" t="s">
         <v>63</v>
       </c>
-      <c r="AF3" t="s">
+      <c r="AG3" t="s">
         <v>57</v>
       </c>
-      <c r="AG3" t="s">
+      <c r="AH3" t="s">
         <v>68</v>
       </c>
-      <c r="AH3" t="s">
+      <c r="AI3" t="s">
         <v>1</v>
       </c>
-      <c r="AI3" t="s">
+      <c r="AJ3" t="s">
         <v>80</v>
       </c>
-      <c r="AJ3" t="s">
-        <v>127</v>
-      </c>
       <c r="AK3" t="s">
+        <v>126</v>
+      </c>
+      <c r="AL3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:38" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1371,41 +1389,41 @@
       <c r="Q4" t="s">
         <v>6</v>
       </c>
-      <c r="S4" t="s">
-        <v>120</v>
-      </c>
-      <c r="V4" t="s">
+      <c r="T4" t="s">
+        <v>119</v>
+      </c>
+      <c r="W4" t="s">
         <v>27</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="AA4" t="s">
         <v>42</v>
       </c>
-      <c r="AB4" t="s">
+      <c r="AC4" t="s">
         <v>55</v>
       </c>
-      <c r="AC4" t="s">
+      <c r="AD4" t="s">
         <v>50</v>
       </c>
-      <c r="AD4" t="s">
+      <c r="AE4" t="s">
         <v>61</v>
       </c>
-      <c r="AE4" t="s">
+      <c r="AF4" t="s">
         <v>62</v>
       </c>
-      <c r="AF4" t="s">
+      <c r="AG4" t="s">
         <v>58</v>
       </c>
-      <c r="AG4" t="s">
+      <c r="AH4" t="s">
         <v>69</v>
       </c>
-      <c r="AI4" t="s">
+      <c r="AJ4" t="s">
         <v>81</v>
       </c>
-      <c r="AJ4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.45">
+      <c r="AK4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="5" spans="1:38" x14ac:dyDescent="0.45">
       <c r="F5" t="s">
         <v>7</v>
       </c>
@@ -1421,91 +1439,91 @@
       <c r="Q5" t="s">
         <v>78</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>28</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AA5" t="s">
         <v>43</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AD5" t="s">
         <v>51</v>
       </c>
-      <c r="AD5" t="s">
+      <c r="AE5" t="s">
         <v>66</v>
       </c>
-      <c r="AE5" t="s">
+      <c r="AF5" t="s">
         <v>64</v>
       </c>
-      <c r="AF5" t="s">
+      <c r="AG5" t="s">
         <v>59</v>
       </c>
-      <c r="AG5" t="s">
+      <c r="AH5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:38" x14ac:dyDescent="0.45">
       <c r="O6" t="s">
         <v>21</v>
       </c>
       <c r="Q6" t="s">
         <v>75</v>
       </c>
-      <c r="V6" t="s">
+      <c r="W6" t="s">
         <v>29</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AA6" t="s">
         <v>44</v>
       </c>
-      <c r="AC6" t="s">
+      <c r="AD6" t="s">
         <v>52</v>
       </c>
-      <c r="AE6" t="s">
+      <c r="AF6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:38" x14ac:dyDescent="0.45">
       <c r="Q7" t="s">
         <v>74</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>30</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="AA7" t="s">
         <v>45</v>
       </c>
-      <c r="AC7" t="s">
+      <c r="AD7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:38" x14ac:dyDescent="0.45">
       <c r="Q8" t="s">
         <v>76</v>
       </c>
-      <c r="V8" t="s">
+      <c r="W8" t="s">
         <v>31</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="AA8" t="s">
         <v>46</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AD8" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.45">
-      <c r="V9" t="s">
+    <row r="9" spans="1:38" x14ac:dyDescent="0.45">
+      <c r="W9" t="s">
         <v>32</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="AA9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.45">
-      <c r="V10" t="s">
+    <row r="10" spans="1:38" x14ac:dyDescent="0.45">
+      <c r="W10" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.45">
-      <c r="V11" t="s">
+    <row r="11" spans="1:38" x14ac:dyDescent="0.45">
+      <c r="W11" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>